<commit_message>
feat: assistente a chat a tutto schermo, documenti di prova completi e parser robusti, riassunto, dossier v4.2 senza consulenza/assicurazioni
- assistente: chat con suggerimenti, scheda ridotta con pillole, colonna di vetro e gradiente giallo
- azienda di prova: modello contabile coerente, bilanci di 16 pagine, visura, cedolini, F24, domanda, business plan, Excel
- lettura documenti veri: importi senza centesimi, un solo blocco di costi, etichette specifiche, F24 per sezioni e crediti, categoria Altro
- nuovo documento Riassunto (7 pagine); dossier v4.2 con la nuova visione; manuale aggiornato

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documenti_di_prova/meridiana_digital_solutions/13_Registro_aiuti_ricevuti.xlsx
+++ b/documenti_di_prova/meridiana_digital_solutions/13_Registro_aiuti_ricevuti.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Registro aiuti" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Domande presentate" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +18,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -46,8 +50,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,148 +418,486 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:J9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ente concedente</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Misura</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Base normativa</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Data concessione</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Data incasso/fruizione</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Importo (EUR)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Regime</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Codice COR (prova)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Impresa unica</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Camera di Commercio di Torino</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Voucher digitalizzazione PMI</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Reg. UE 2023/2831</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2024-04-12</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2024-09-30</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>10000</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>de minimis</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>COR-0000001</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Meridiana Digital Solutions S.r.l.</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Spese di consulenza e licenze 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Regione Piemonte</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Contributo partecipazione fiere</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Reg. UE 2023/2831</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2025-10-03</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2025-12-15</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>6500</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>de minimis</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>COR-0000002</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Meridiana Digital Solutions S.r.l.</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Fiera di settore a Milano, 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Agenzia delle Entrate</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Credito d'imposta ricerca e sviluppo 2023</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Art. 1 c. 198 L. 160/2019</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2024-06-30</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2024-07-16</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>12000</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>credito d'imposta (esenzione)</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Meridiana Digital Solutions S.r.l.</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Compensazione in F24, codice tributo 6938</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Agenzia delle Entrate</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Credito d'imposta ricerca e sviluppo 2024</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Art. 1 c. 198 L. 160/2019</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2025-06-30</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2025-07-16</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>31500</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>credito d'imposta (esenzione)</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Meridiana Digital Solutions S.r.l.</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Compensazione in F24, codice tributo 6938</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Agenzia delle Entrate</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Credito d'imposta ricerca e sviluppo 2025</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Art. 1 c. 198 L. 160/2019</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>42000</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>credito d'imposta (esenzione)</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Meridiana Digital Solutions S.r.l.</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Compensazione in F24, codice tributo 6938</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Totale de minimis nel triennio</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8">
+        <f>SUM(F2:F3)</f>
+        <v/>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Massimale 300.000 EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Margine residuo</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9">
+        <f>300000-F7</f>
+        <v/>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Ente concedente</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Misura</t>
+          <t>Ente</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Base normativa</t>
+          <t>Bando</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Data concessione</t>
+          <t>Importo richiesto (EUR)</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Importo (EUR)</t>
+          <t>Esito</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Regime</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Codice COR (prova)</t>
+          <t>Note</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>Camera di Commercio di Torino</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Voucher digitalizzazione PMI</t>
-        </is>
-      </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Reg. UE 2831/2024</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2024-04-12</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>10000</v>
+          <t>Voucher digitalizzazione 2026</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>12000</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>In istruttoria</t>
+        </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>de minimis</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>COR-0000001</t>
+          <t>Presentata via PEC</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>Regione Piemonte</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Contributo partecipazione fiere</t>
-        </is>
-      </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Reg. UE 2831/2024</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>2025-10-03</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>6500</v>
+          <t>Bando SWIch 2026</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>140000</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Non presentata</t>
+        </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>de minimis</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>COR-0000002</t>
+          <t>Verifica dei requisiti in corso</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Agenzia delle Entrate</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Credito d'imposta ricerca e sviluppo 2025</t>
+          <t>Invitalia</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Art. 1 c. 198 L. 160/2019</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>2026-06-30</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>42000</v>
+          <t>Smart&amp;Start Italia</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Non ammissibile</t>
+        </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>credito d'imposta</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>L'impresa ha più di 5 anni dall'iscrizione</t>
         </is>
       </c>
     </row>

</xml_diff>